<commit_message>
F: feedback from xiaolong accepted
</commit_message>
<xml_diff>
--- a/tests/test_plan_v1.1.xlsx
+++ b/tests/test_plan_v1.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/minhakim/Project/glucolink-a2/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81F77DAC-9E6F-C948-A999-CA1B33E37263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAD24410-6096-BF41-9FEE-73A2962C140B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10820" yWindow="680" windowWidth="23740" windowHeight="19940" activeTab="1" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
+    <workbookView xWindow="17280" yWindow="680" windowWidth="17280" windowHeight="19940" xr2:uid="{38C2F623-CE48-954F-9147-651889642CF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Plan v1.1" sheetId="1" r:id="rId1"/>
@@ -39,40 +39,8 @@
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="2">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="2">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="294">
   <si>
     <t>Test ID</t>
   </si>
@@ -369,9 +337,6 @@
   </si>
   <si>
     <t>status</t>
-  </si>
-  <si>
-    <t>SELECT * FROM reporting.vw_uc1_care_gaps WHERE patient_id = 'GL-0001'</t>
   </si>
   <si>
     <t>SELECT covered_days, pdc, adherence_status FROM reporting.vw_uc2_pdc WHERE patient_id = 'GL-0002';</t>
@@ -437,9 +402,6 @@
          count(*) FILTER (WHERE patient_id ~ '^GL-[0-9]{4}$') AS well_formed,
          count(*) FILTER (WHERE home_clinic_key IS NULL)      AS null_home_clinic
   FROM curated.dim_patient;</t>
-  </si>
-  <si>
-    <t>Pass</t>
   </si>
   <si>
     <t>U103</t>
@@ -631,16 +593,6 @@
   </si>
   <si>
     <t>The three excluded messages are the intended ones, identified by message_id: MSG-0022 REJECTED_UNIT (blank unit kept as '', no converted value), MSG-0025 FUTURE_DATE (collected 2026-10-01, after the as-of date), MSG-0032 DUPLICATE (second message for OBS-0031) while MSG-0031 stays VALID.</t>
-  </si>
-  <si>
-    <t>MSG-0022 OBS-0022 REJECTED_UNIT unit '' hba1c NULL | MSG-0025 OBS-0025 FUTURE_DATE | 
-    MSG-0031 OBS-0031 VALID | MSG-0032 OBS-0031 DUPLICATE</t>
-  </si>
-  <si>
-    <t>SELECT message_id, observation_id, dq_status, unit_as_received, hba1c_mmol_mol, collected_date
-  FROM cleansed.lab_result
-  WHERE message_id IN ('MSG-0022','MSG-0025','MSG-0031','MSG-0032')
-  ORDER BY message_id;</t>
   </si>
   <si>
     <t>Matching quality against audit.identity_truth (read only after matching): precision = correct LINKED lab/pharmacy links / all LINKED lab/pharmacy links; recall = correct links /lab/pharmacy records whose true person has a GP record. A link is correct when the record's true person is the true person of the GP record(s) behind the same patient_id.</t>
@@ -793,7 +745,311 @@
     <t>After run 2: tests = passed (all rows of audit.test_result), failed 0; raw_runs 2; all layer counts identical to run 1</t>
   </si>
   <si>
-    <t>/-- Post the Teams warning (D9), run 01 -&gt; 02 -&gt; 02b again on the test database, then:
+    <t>SELECT count(*) AS n_rows
+  FROM reporting.vw_uc4_care_path_breaks
+  WHERE detail LIKE '%OBS-0031%' OR detail LIKE '%MSG-0032%' OR patient_id = 'GL-0009';</t>
+  </si>
+  <si>
+    <t>n_rows 0</t>
+  </si>
+  <si>
+    <t>P13 Chloe White, P09 Grace Taylor</t>
+  </si>
+  <si>
+    <t>SELECT count(*) AS n_rows FROM reporting.vw_uc1_care_gaps WHERE patient_id IN ('GL-0013', 'GL-0009');</t>
+  </si>
+  <si>
+    <t>03_raw_extract.sql copies every source table unchanged: each of the 11 raw.* tables has the same row count as its src_* table.</t>
+  </si>
+  <si>
+    <t>P11 Emily Davis, P03 Ahmed Khan</t>
+  </si>
+  <si>
+    <t>NEGATIVE - results outside the window are excluded: P11's FUTURE_DATE result (OBS-0025, 2026-10-01) is ignored so 54.0 -&gt; 50.0 is STABLE (-4.0); P03's 2025-06-10 result is before 2025-09-01 so only one result remains, INSUFFICIENT_HISTORY.</t>
+  </si>
+  <si>
+    <t>GL-0003 n_results 1 change NULL INSUFFICIENT_HISTORY | GL-0011 n_results 2 54.0 -&gt; 50.0 change -4.0 STABLE</t>
+  </si>
+  <si>
+    <t>SELECT patient_id, n_results, first_hba1c, last_hba1c, change_mmol_mol, trend_status
+  FROM reporting.vw_uc3_hba1c_trend
+  WHERE patient_id IN ('GL-0003','GL-0011')
+  ORDER BY patient_id;</t>
+  </si>
+  <si>
+    <t>How we check (runnable SQL)</t>
+  </si>
+  <si>
+    <t>Due</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>File name (evidence/)</t>
+  </si>
+  <si>
+    <t>What the screenshot must show</t>
+  </si>
+  <si>
+    <t>Received</t>
+  </si>
+  <si>
+    <t>Checked by F (date)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Evidence rules (evidence/README.md)</t>
+  </si>
+  <si>
+    <t>2. Each screenshot shows the query, the result grid AND the database name (CloudBeaver connection shown in the header).</t>
+  </si>
+  <si>
+    <t>3. One screenshot per acceptance check, uploaded to evidence/ by the owner from their own GitHub account, then posted in Teams with the file name.</t>
+  </si>
+  <si>
+    <t>1. File name: YYYY-MM-DD_&lt;package letter&gt;_&lt;what&gt;.png, e.g. 2026-10-08_C_raw_counts.png.</t>
+  </si>
+  <si>
+    <t>4. F keeps this list up to date daily and reminds owners in Teams the evening before each due time.</t>
+  </si>
+  <si>
+    <t>run result</t>
+  </si>
+  <si>
+    <t>C
+Quang</t>
+  </si>
+  <si>
+    <t>2026-10-07
+(12:00)</t>
+  </si>
+  <si>
+    <t>B
+Zhihao</t>
+  </si>
+  <si>
+    <t>D
+Yutong</t>
+  </si>
+  <si>
+    <t>E
+Shuo</t>
+  </si>
+  <si>
+    <t>F
+Minha</t>
+  </si>
+  <si>
+    <t>B+F</t>
+  </si>
+  <si>
+    <t>C-2</t>
+  </si>
+  <si>
+    <t>B-1</t>
+  </si>
+  <si>
+    <t>D-1</t>
+  </si>
+  <si>
+    <t>D-2</t>
+  </si>
+  <si>
+    <t>B-2</t>
+  </si>
+  <si>
+    <t>C-3</t>
+  </si>
+  <si>
+    <t>D-3</t>
+  </si>
+  <si>
+    <t>E-2</t>
+  </si>
+  <si>
+    <t>F-3</t>
+  </si>
+  <si>
+    <t>E-3</t>
+  </si>
+  <si>
+    <t>D-4</t>
+  </si>
+  <si>
+    <t>E-4</t>
+  </si>
+  <si>
+    <t>F-4</t>
+  </si>
+  <si>
+    <t>F-5</t>
+  </si>
+  <si>
+    <t>2026-10-07_C_source_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-07
+(21:00)</t>
+  </si>
+  <si>
+    <t>2026-10-07
+(23:00)</t>
+  </si>
+  <si>
+    <t>2026-10-08
+(12:00)</t>
+  </si>
+  <si>
+    <t>2026-10-08
+(21:00)</t>
+  </si>
+  <si>
+    <t>2026-10-09
+(12:00)</t>
+  </si>
+  <si>
+    <t>2026-10-09
+(18:00)</t>
+  </si>
+  <si>
+    <t>2026-10-10
+(12:00)</t>
+  </si>
+  <si>
+    <t>2026-10-09
+(21:00)</t>
+  </si>
+  <si>
+    <t>2026-10-11
+(15:00)</t>
+  </si>
+  <si>
+    <t>2026-10-11
+(18:00)</t>
+  </si>
+  <si>
+    <t>2026-10-10
+(21:00)</t>
+  </si>
+  <si>
+    <t>2026-10-07_B_setup_check.png</t>
+  </si>
+  <si>
+    <t>01 fix+48 patient records: gp_patient 18, lab_patient 17, pharmacy_patient 13</t>
+  </si>
+  <si>
+    <t>00_setup.sql: rule_parameter shows the 9 D1 names and values</t>
+  </si>
+  <si>
+    <t>encounter 28, dispense 68, identity_truth 48</t>
+  </si>
+  <si>
+    <t>Card D four-row query (GP-0001, PATH0001, PH-1001, PH-1014) + total 48 (18/17/13)</t>
+  </si>
+  <si>
+    <t>patient_master 17; match_status LINKED 46 / REVIEW 1 / UNMATCHED 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 02b loaded: observation_message 36, result_delivery 34 </t>
+  </si>
+  <si>
+    <t>11 raw tables next to source counts (all equal); pipeline_run latest SUCCESS, 225</t>
+  </si>
+  <si>
+    <t>dq_status VALID 33 / DUPLICATE 1 / REJECTED_UNIT 1 / FUTURE_DATE 1; OBS-0001 dates 2025-10-10 / 2025-10-11; encounter 28, dispense 68</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dim_patient 17 rows, no NULL home_clinic_key, Sarah Lee -&gt; Parramatta Family Practice (file name suggested by F) </t>
+  </si>
+  <si>
+    <t>Metabase query on the reporting schema (or note that the Excel fallback starts Fri 9 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fact_encounter 28, fact_lab_result 32, fact_dispense 65; distinct event ids = rows </t>
+  </si>
+  <si>
+    <t xml:space="preserve">vw_uc2_pdc 11 rows with the card D-4 PDC values </t>
+  </si>
+  <si>
+    <t xml:space="preserve">vw_uc1_care_gaps 8 rows; vw_uc3_hba1c_trend 16 rows, no NULL rising_despite_adherence  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">vw_uc4_care_path_breaks 2 rows (Olivia Brown RESULT_NOT_RETURNED, James Wilson MULTI_PHARMACY_OVERLAP) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">09_tests.sql summary: count() = count() FILTER (WHERE passed), &gt;= 30, 0 failed  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The three (or more) dashboards showing 8 / 11/ 16 / 2   </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full 00 -&gt; 10 run on glucolink_a2_test: layer  counts and test summary after run 2  </t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>2026-10-07_C_part2_counts.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2026-10-07_D_patient_record.png</t>
+  </si>
+  <si>
+    <t>2026-10-07_D_identity_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-07_B_02b_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-08_C_raw_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-08_D_lab_result_dq.png</t>
+  </si>
+  <si>
+    <t>2026-10-08_E_dim_patient.png</t>
+  </si>
+  <si>
+    <t>2026-10-08_F_dashboard_tool.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2026-10-09_E_fact_counts.png</t>
+  </si>
+  <si>
+    <t>2026-10-09_D_vw_uc2.png</t>
+  </si>
+  <si>
+    <t>2026-10-09_E_vw_uc1_uc3.png</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2026-10-10_D_vw_uc4.png</t>
+  </si>
+  <si>
+    <t>2026-10-10_F_test_results.png</t>
+  </si>
+  <si>
+    <t>2026-10-11_F_dashboards.png</t>
+  </si>
+  <si>
+    <t>2026-10-11_BF_full_rerun.png</t>
+  </si>
+  <si>
+    <t>C-1</t>
+  </si>
+  <si>
+    <t>Not run</t>
+  </si>
+  <si>
+    <t>-- Post the Teams warning (D9), run 01 -&gt; 02 -&gt; 02b again on the test database, then:
   SELECT (SELECT count(*) FROM src_gp.gp_patient) AS gp_patient,
          (SELECT count(*) FROM src_gp.encounter) AS encounter,
          (SELECT count(*) FROM src_lab.observation_message) AS observation_message,
@@ -801,264 +1057,26 @@
          (SELECT count(*) FROM src_pharm.dispense) AS dispense;</t>
   </si>
   <si>
-    <t xml:space="preserve"> /-- After the second full 00 -&gt; 10 run on glucolink_a2_test:
+    <t>-- After the second full 00 -&gt; 10 run on glucolink_a2_test:
   SELECT (SELECT count(*) FROM audit.test_result) AS tests,
          (SELECT count(*) FROM audit.test_result WHERE passed) AS passed,
          (SELECT count(*) FROM audit.test_result WHERE NOT passed) AS failed,
          (SELECT count(*) FROM audit.pipeline_run WHERE pipeline_name = '03_raw_extract') AS raw_runs;</t>
   </si>
   <si>
-    <t>SELECT count(*) AS n_rows
-  FROM reporting.vw_uc4_care_path_breaks
-  WHERE detail LIKE '%OBS-0031%' OR detail LIKE '%MSG-0032%' OR patient_id = 'GL-0009';</t>
-  </si>
-  <si>
-    <t>n_rows 0</t>
-  </si>
-  <si>
-    <t>P13 Chloe White, P09 Grace Taylor</t>
-  </si>
-  <si>
-    <t>SELECT count(*) AS n_rows FROM reporting.vw_uc1_care_gaps WHERE patient_id IN ('GL-0013', 'GL-0009');</t>
-  </si>
-  <si>
-    <t>03_raw_extract.sql copies every source table unchanged: each of the 11 raw.* tables has the same row count as its src_* table.</t>
-  </si>
-  <si>
-    <t>P11 Emily Davis, P03 Ahmed Khan</t>
-  </si>
-  <si>
-    <t>NEGATIVE - results outside the window are excluded: P11's FUTURE_DATE result (OBS-0025, 2026-10-01) is ignored so 54.0 -&gt; 50.0 is STABLE (-4.0); P03's 2025-06-10 result is before 2025-09-01 so only one result remains, INSUFFICIENT_HISTORY.</t>
-  </si>
-  <si>
-    <t>GL-0003 n_results 1 change NULL INSUFFICIENT_HISTORY | GL-0011 n_results 2 54.0 -&gt; 50.0 change -4.0 STABLE</t>
-  </si>
-  <si>
-    <t>SELECT patient_id, n_results, first_hba1c, last_hba1c, change_mmol_mol, trend_status
-  FROM reporting.vw_uc3_hba1c_trend
-  WHERE patient_id IN ('GL-0003','GL-0011')
-  ORDER BY patient_id;</t>
-  </si>
-  <si>
-    <t>How we check (runnable SQL)</t>
-  </si>
-  <si>
-    <t>Due</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>Card</t>
-  </si>
-  <si>
-    <t>File name (evidence/)</t>
-  </si>
-  <si>
-    <t>What the screenshot must show</t>
-  </si>
-  <si>
-    <t>Received</t>
-  </si>
-  <si>
-    <t>Checked by F (date)</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Evidence rules (evidence/README.md)</t>
-  </si>
-  <si>
-    <t>2. Each screenshot shows the query, the result grid AND the database name (CloudBeaver connection shown in the header).</t>
-  </si>
-  <si>
-    <t>3. One screenshot per acceptance check, uploaded to evidence/ by the owner from their own GitHub account, then posted in Teams with the file name.</t>
-  </si>
-  <si>
-    <t>1. File name: YYYY-MM-DD_&lt;package letter&gt;_&lt;what&gt;.png, e.g. 2026-10-08_C_raw_counts.png.</t>
-  </si>
-  <si>
-    <t>4. F keeps this list up to date daily and reminds owners in Teams the evening before each due time.</t>
-  </si>
-  <si>
-    <t>run result</t>
-  </si>
-  <si>
-    <t>C
-Quang</t>
-  </si>
-  <si>
-    <t>2026-10-07
-(12:00)</t>
-  </si>
-  <si>
-    <t>B
-Zhihao</t>
-  </si>
-  <si>
-    <t>D
-Yutong</t>
-  </si>
-  <si>
-    <t>E
-Shuo</t>
-  </si>
-  <si>
-    <t>F
-Minha</t>
-  </si>
-  <si>
-    <t>B+F</t>
-  </si>
-  <si>
-    <t>C-2</t>
-  </si>
-  <si>
-    <t>B-1</t>
-  </si>
-  <si>
-    <t>D-1</t>
-  </si>
-  <si>
-    <t>D-2</t>
-  </si>
-  <si>
-    <t>B-2</t>
-  </si>
-  <si>
-    <t>C-3</t>
-  </si>
-  <si>
-    <t>D-3</t>
-  </si>
-  <si>
-    <t>E-2</t>
-  </si>
-  <si>
-    <t>F-3</t>
-  </si>
-  <si>
-    <t>E-3</t>
-  </si>
-  <si>
-    <t>D-4</t>
-  </si>
-  <si>
-    <t>E-4</t>
-  </si>
-  <si>
-    <t>F-4</t>
-  </si>
-  <si>
-    <t>F-5</t>
-  </si>
-  <si>
-    <t>2026-10-07_C_source_counts.png</t>
-  </si>
-  <si>
-    <t>2026-10-07
-(21:00)</t>
-  </si>
-  <si>
-    <t>2026-10-07
-(23:00)</t>
-  </si>
-  <si>
-    <t>2026-10-08
-(12:00)</t>
-  </si>
-  <si>
-    <t>2026-10-08
-(21:00)</t>
-  </si>
-  <si>
-    <t>2026-10-09
-(12:00)</t>
-  </si>
-  <si>
-    <t>2026-10-09
-(18:00)</t>
-  </si>
-  <si>
-    <t>2026-10-10
-(12:00)</t>
-  </si>
-  <si>
-    <t>2026-10-09
-(21:00)</t>
-  </si>
-  <si>
-    <t>2026-10-11
-(15:00)</t>
-  </si>
-  <si>
-    <t>2026-10-11
-(18:00)</t>
-  </si>
-  <si>
-    <t>2026-10-10
-(21:00)</t>
-  </si>
-  <si>
-    <t>2026-10-07_B_setup_check.png</t>
-  </si>
-  <si>
-    <t>01 fix+48 patient records: gp_patient 18, lab_patient 17, pharmacy_patient 13</t>
-  </si>
-  <si>
-    <t>00_setup.sql: rule_parameter shows the 9 D1 names and values</t>
-  </si>
-  <si>
-    <t>encounter 28, dispense 68, identity_truth 48</t>
-  </si>
-  <si>
-    <t>Card D four-row query (GP-0001, PATH0001, PH-1001, PH-1014) + total 48 (18/17/13)</t>
-  </si>
-  <si>
-    <t>patient_master 17; match_status LINKED 46 / REVIEW 1 / UNMATCHED 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 02b loaded: observation_message 36, result_delivery 34 </t>
-  </si>
-  <si>
-    <t>11 raw tables next to source counts (all equal); pipeline_run latest SUCCESS, 225</t>
-  </si>
-  <si>
-    <t>dq_status VALID 33 / DUPLICATE 1 / REJECTED_UNIT 1 / FUTURE_DATE 1; OBS-0001 dates 2025-10-10 / 2025-10-11; encounter 28, dispense 68</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dim_patient 17 rows, no NULL home_clinic_key, Sarah Lee -&gt; Parramatta Family Practice (file name suggested by F) </t>
-  </si>
-  <si>
-    <t>Metabase query on the reporting schema (or note that the Excel fallback starts Fri 9 Oct)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fact_encounter 28, fact_lab_result 32, fact_dispense 65; distinct event ids = rows </t>
-  </si>
-  <si>
-    <t xml:space="preserve">vw_uc2_pdc 11 rows with the card D-4 PDC values </t>
-  </si>
-  <si>
-    <t xml:space="preserve">vw_uc1_care_gaps 8 rows; vw_uc3_hba1c_trend 16 rows, no NULL rising_despite_adherence  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">vw_uc4_care_path_breaks 2 rows (Olivia Brown RESULT_NOT_RETURNED, James Wilson MULTI_PHARMACY_OVERLAP) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">09_tests.sql summary: count() = count() FILTER (WHERE passed), &gt;= 30, 0 failed  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">The three (or more) dashboards showing 8 / 11/ 16 / 2   </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full 00 -&gt; 10 run on glucolink_a2_test: layer  counts and test summary after run 2  </t>
-  </si>
-  <si>
-    <t>Y</t>
-  </si>
-  <si>
-    <t>N</t>
+    <t>SELECT * FROM reporting.vw_uc1_care_gaps WHERE patient_id = 'GL-0001';</t>
+  </si>
+  <si>
+    <t>SELECT message_id, observation_id, dq_status, unit_as_received,
+         (unit_as_received = '') AS unit_is_empty_string,
+         hba1c_mmol_mol, collected_date
+  FROM cleansed.lab_result
+  WHERE message_id IN ('MSG-0022','MSG-0025','MSG-0031','MSG-0032')
+  ORDER BY message_id;</t>
+  </si>
+  <si>
+    <t>MSG-0022 OBS-0022 REJECTED_UNIT unit '' unit_is_empty_string true hba1c NULL | MSG-0025 OBS-0025 FUTURE_DATE | 
+    MSG-0031 OBS-0031 VALID | MSG-0032 OBS-0031 DUPLICATE</t>
   </si>
 </sst>
 </file>
@@ -1163,7 +1181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1221,19 +1239,52 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="11">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1254,6 +1305,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1287,6 +1348,16 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1298,75 +1369,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="2">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1713,13 +1715,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>98</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1739,7 +1741,10 @@
         <v>66</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>187</v>
+        <v>183</v>
+      </c>
+      <c r="G2" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1759,7 +1764,10 @@
         <v>68</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>188</v>
+        <v>184</v>
+      </c>
+      <c r="G3" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1779,7 +1787,10 @@
         <v>70</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>189</v>
+        <v>185</v>
+      </c>
+      <c r="G4" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="68" x14ac:dyDescent="0.2">
@@ -1796,10 +1807,13 @@
         <v>71</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>191</v>
+        <v>187</v>
+      </c>
+      <c r="G5" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="238" x14ac:dyDescent="0.2">
@@ -1813,18 +1827,21 @@
         <v>42</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+      <c r="G6" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>34</v>
@@ -1833,24 +1850,21 @@
         <v>42</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="F7" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="H7" t="e" vm="1">
-        <v>#VALUE!</v>
+        <v>108</v>
+      </c>
+      <c r="G7" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>34</v>
@@ -1859,13 +1873,16 @@
         <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="F8" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>108</v>
+      <c r="G8" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1885,12 +1902,15 @@
         <v>72</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>194</v>
+        <v>190</v>
+      </c>
+      <c r="G9" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>34</v>
@@ -1899,24 +1919,21 @@
         <v>42</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="2" t="s">
-        <v>113</v>
-      </c>
       <c r="G10" t="s">
-        <v>118</v>
-      </c>
-      <c r="H10" t="e" vm="2">
-        <v>#VALUE!</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>34</v>
@@ -1925,33 +1942,39 @@
         <v>43</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="F11" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>117</v>
+      <c r="G11" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="68" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>143</v>
+      <c r="G12" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.2">
@@ -1973,6 +1996,9 @@
       <c r="F13" s="4" t="s">
         <v>75</v>
       </c>
+      <c r="G13" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
@@ -1993,6 +2019,9 @@
       <c r="F14" s="4" t="s">
         <v>78</v>
       </c>
+      <c r="G14" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
@@ -2005,56 +2034,65 @@
         <v>44</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>169</v>
+        <v>293</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>170</v>
+        <v>292</v>
+      </c>
+      <c r="G15" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="85" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C16" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G16" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>151</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="85" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C17" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="G17" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
@@ -2073,28 +2111,34 @@
       <c r="F18" s="4" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C19" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G19" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A20" s="6" t="s">
         <v>15</v>
       </c>
@@ -2113,8 +2157,11 @@
       <c r="F20" s="4" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G20" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A21" s="6" t="s">
         <v>16</v>
       </c>
@@ -2133,8 +2180,11 @@
       <c r="F21" s="4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+      <c r="G21" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>17</v>
       </c>
@@ -2145,16 +2195,19 @@
         <v>47</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>171</v>
+      </c>
+      <c r="G22" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>18</v>
       </c>
@@ -2162,19 +2215,22 @@
         <v>36</v>
       </c>
       <c r="C23" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E23" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G23" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A24" s="6" t="s">
         <v>19</v>
       </c>
@@ -2185,16 +2241,19 @@
         <v>49</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+      <c r="G24" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A25" s="6" t="s">
         <v>20</v>
       </c>
@@ -2205,36 +2264,42 @@
         <v>50</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="G25" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B26" s="9" t="s">
         <v>36</v>
       </c>
       <c r="C26" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E26" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="404" x14ac:dyDescent="0.2">
+      <c r="G26" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="404" x14ac:dyDescent="0.2">
       <c r="A27" s="6" t="s">
         <v>21</v>
       </c>
@@ -2245,16 +2310,19 @@
         <v>43</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+      <c r="G27" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A28" s="6" t="s">
         <v>22</v>
       </c>
@@ -2271,10 +2339,13 @@
         <v>85</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+      <c r="G28" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>23</v>
       </c>
@@ -2282,21 +2353,24 @@
         <v>37</v>
       </c>
       <c r="C29" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E29" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+      <c r="G29" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B30" s="10" t="s">
         <v>37</v>
@@ -2311,30 +2385,36 @@
         <v>86</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="34" x14ac:dyDescent="0.2">
+        <v>291</v>
+      </c>
+      <c r="G30" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A31" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B31" s="10" t="s">
         <v>37</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>58</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>198</v>
+      </c>
+      <c r="G31" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A32" s="6" t="s">
         <v>24</v>
       </c>
@@ -2353,8 +2433,11 @@
       <c r="F32" s="4" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="G32" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A33" s="6" t="s">
         <v>25</v>
       </c>
@@ -2362,19 +2445,22 @@
         <v>38</v>
       </c>
       <c r="C33" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="F33" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="E33" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G33" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A34" s="6" t="s">
         <v>26</v>
       </c>
@@ -2391,12 +2477,15 @@
         <v>89</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+      <c r="G34" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A35" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B35" s="10" t="s">
         <v>38</v>
@@ -2408,13 +2497,16 @@
         <v>61</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="G35" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A36" s="6" t="s">
         <v>27</v>
       </c>
@@ -2433,8 +2525,11 @@
       <c r="F36" s="4" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+      <c r="G36" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A37" s="6" t="s">
         <v>28</v>
       </c>
@@ -2442,21 +2537,24 @@
         <v>39</v>
       </c>
       <c r="C37" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="F37" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G37" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A38" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B38" s="10" t="s">
         <v>39</v>
@@ -2471,10 +2569,13 @@
         <v>92</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+        <v>100</v>
+      </c>
+      <c r="G38" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A39" s="6" t="s">
         <v>29</v>
       </c>
@@ -2482,39 +2583,45 @@
         <v>39</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+        <v>203</v>
+      </c>
+      <c r="G39" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A40" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B40" s="10" t="s">
         <v>39</v>
       </c>
       <c r="C40" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="E40" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="F40" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="E40" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G40" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A41" s="6" t="s">
         <v>30</v>
       </c>
@@ -2525,16 +2632,19 @@
         <v>97</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+      <c r="G41" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A42" s="6" t="s">
         <v>31</v>
       </c>
@@ -2548,13 +2658,16 @@
         <v>64</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+        <v>195</v>
+      </c>
+      <c r="G42" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
         <v>32</v>
       </c>
@@ -2570,11 +2683,14 @@
       <c r="E43" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F43" s="2" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="F43" s="21" t="s">
+        <v>289</v>
+      </c>
+      <c r="G43" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
         <v>33</v>
       </c>
@@ -2588,19 +2704,22 @@
         <v>95</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+      <c r="F44" s="21" t="s">
+        <v>290</v>
+      </c>
+      <c r="G44" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D45" s="2"/>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D46" s="2"/>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="D47" s="2"/>
     </row>
     <row r="49" spans="4:4" x14ac:dyDescent="0.2">
@@ -2609,17 +2728,42 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="6" operator="equal">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
       <formula>"Fail"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="1">
+  <conditionalFormatting sqref="G2:G7">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
+      <formula>"Not run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+      <formula>"Not run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"Not run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:G44">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>"Not run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"Not run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1048576" xr:uid="{8DF08CFE-93BA-2846-90B2-153942F105FA}">
       <formula1>"Not run, Pass, Fail, Blocked"</formula1>
     </dataValidation>
@@ -2642,7 +2786,7 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -2658,7 +2802,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B2" s="15"/>
       <c r="C2" s="15"/>
@@ -2674,7 +2818,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="15"/>
@@ -2690,7 +2834,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
@@ -2706,7 +2850,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -2722,108 +2866,117 @@
     </row>
     <row r="9" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="E9" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>211</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="H9" s="18" t="s">
         <v>212</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="E9" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>216</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>217</v>
-      </c>
-      <c r="H9" s="18" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="16" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C10" t="s">
-        <v>232</v>
+        <v>287</v>
       </c>
       <c r="D10" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>277</v>
+        <v>270</v>
+      </c>
+      <c r="G10" s="20">
+        <v>46303</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" s="16" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B11" s="16" t="s">
+        <v>221</v>
+      </c>
+      <c r="C11" t="s">
         <v>227</v>
       </c>
-      <c r="C11" t="s">
-        <v>233</v>
-      </c>
       <c r="D11" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>277</v>
+        <v>270</v>
+      </c>
+      <c r="G11" s="20">
+        <v>46303</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A12" s="16" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C12" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="D12" t="s">
-        <v>246</v>
+        <v>272</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>277</v>
+        <v>270</v>
+      </c>
+      <c r="G12" s="20">
+        <v>46303</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" s="16" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B13" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="C13" t="s">
         <v>228</v>
       </c>
-      <c r="C13" t="s">
-        <v>234</v>
-      </c>
       <c r="D13" t="s">
-        <v>246</v>
+        <v>273</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="G13" s="20">
         <v>46302</v>
@@ -2831,22 +2984,22 @@
     </row>
     <row r="14" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C14" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="D14" t="s">
-        <v>246</v>
+        <v>274</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="G14" s="20">
         <v>46302</v>
@@ -2854,206 +3007,218 @@
     </row>
     <row r="15" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A15" s="16" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C15" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="D15" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>264</v>
+        <v>258</v>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>270</v>
+      </c>
+      <c r="G15" s="20">
+        <v>46303</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" s="16" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C16" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="D16" t="s">
-        <v>246</v>
+        <v>276</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>265</v>
+        <v>259</v>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>270</v>
+      </c>
+      <c r="G16" s="20">
+        <v>46303</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="68" x14ac:dyDescent="0.2">
       <c r="A17" s="16" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C17" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="D17" t="s">
-        <v>246</v>
+        <v>277</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A18" s="16" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C18" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D18" t="s">
-        <v>246</v>
+        <v>278</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A19" s="16" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="D19" t="s">
-        <v>246</v>
+        <v>279</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" s="16" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C20" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="D20" t="s">
-        <v>246</v>
+        <v>280</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A21" s="16" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C21" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D21" t="s">
-        <v>246</v>
+        <v>281</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" s="16" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C22" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="D22" t="s">
-        <v>246</v>
+        <v>282</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" s="17" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="C23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="D23" t="s">
-        <v>246</v>
+        <v>283</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" s="17" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C24" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="D24" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" s="16" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C25" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="D25" t="s">
-        <v>246</v>
+        <v>285</v>
       </c>
       <c r="E25" s="16" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" s="16" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C26" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="D26" t="s">
-        <v>246</v>
+        <v>286</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -3065,11 +3230,11 @@
     <mergeCell ref="A1:L1"/>
   </mergeCells>
   <conditionalFormatting sqref="F10:F26">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="1" operator="equal">
+      <formula>"N"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
       <formula>"Y"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
-      <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>